<commit_message>
prev1.1.4 update, including a lot of bugfixes
</commit_message>
<xml_diff>
--- a/docs/DevelopHistoryAndPlan.xlsx
+++ b/docs/DevelopHistoryAndPlan.xlsx
@@ -14,9 +14,9 @@
     <sheet name="长期约定" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'维护说明'!$B$4:$D$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'维护说明'!$B$4:$D$25</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'版本速查'!$B$4:$I$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'计划与企划'!$B$4:$F$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'计划与企划'!$B$4:$G$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'长期约定'!$B$4:$C$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="B2:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -845,8 +845,76 @@
         </is>
       </c>
     </row>
+    <row r="22" ht="38" customHeight="1">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Temp.txt 规则</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>章节行</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>版本行(如 `v1.1.4企划部分:`)-&gt; 决定「目标版本」;整份没有版本行则记 未定 / 企划池。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>Temp.txt 规则</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>负责人行</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>`RoF负责:` -&gt; 决定「负责人」;行尾括号内文字会记进「关联 / 备注」。</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Temp.txt 规则</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>条目行</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>`1.` / `-` / `*` 开头各成一条;不带头标记的续行并入上一条。</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="38" customHeight="1">
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Temp.txt 规则</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>入库方式</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>运行 tools/notes_organizer.py:条目写进「计划与企划」,重复条目自动跳过,原文存 docs/notes_archive/ 后清空 Temp.txt。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="B4:D21"/>
+  <autoFilter ref="B4:D25"/>
   <mergeCells count="1">
     <mergeCell ref="B2:D2"/>
   </mergeCells>
@@ -860,7 +928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="B2:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1125,7 +1193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D47"/>
+  <dimension ref="B2:D47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1166,8 +1234,6 @@
           <t>未发布 · 开发中(mergeServerPromote)· 9 个提交 · 202609102126 → 202609111223</t>
         </is>
       </c>
-      <c r="C5" s="9" t="n"/>
-      <c r="D5" s="9" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="B6" s="5" t="inlineStr">
@@ -1328,8 +1394,6 @@
           <t>v1.1.3 · 体验与稳定修补 · 已发布 · 锚点 6f83352 @ 202609101150 · 10 个提交</t>
         </is>
       </c>
-      <c r="C15" s="9" t="n"/>
-      <c r="D15" s="9" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="B16" s="6" t="inlineStr">
@@ -1507,8 +1571,6 @@
           <t>v1.1.2 · 玩法大版本 · 已发布 · 锚点 5043a50 @ 202609091707 · 19 个提交</t>
         </is>
       </c>
-      <c r="C26" s="9" t="n"/>
-      <c r="D26" s="9" t="n"/>
     </row>
     <row r="27" ht="54" customHeight="1">
       <c r="B27" s="6" t="inlineStr">
@@ -1839,8 +1901,6 @@
           <t>v1.1.1 · 基线快照 · 已发布 · 锚点 0232a0d @ 202609071321 · 此前 316 个提交(原作者 280 + 本仓 36),整体作为起点不逐条展开</t>
         </is>
       </c>
-      <c r="C46" s="9" t="n"/>
-      <c r="D46" s="9" t="n"/>
     </row>
     <row r="47" ht="38" customHeight="1">
       <c r="B47" s="5" t="inlineStr">
@@ -1877,15 +1937,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="B2:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="54" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="54" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -1910,15 +1971,20 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>负责人</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
           <t>状态</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>条目</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>关联 / 备注</t>
         </is>
@@ -1935,17 +2001,18 @@
           <t>v1.1.4</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="F5" s="3" t="inlineStr">
         <is>
           <t>换弹进 PvP/大乱斗:R 边沿进输入包 + 服务端权威弹夹 + 弹量随快照镜像(三件套)</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="n"/>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
@@ -1958,17 +2025,18 @@
           <t>v1.1.4</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>大乱斗公网可用:先试 Tailscale/ZeroTier 组网,再评估轻量云自建服</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr"/>
+      <c r="G6" s="4" t="n"/>
     </row>
     <row r="7" ht="38" customHeight="1">
       <c r="B7" s="3" t="inlineStr">
@@ -1981,17 +2049,18 @@
           <t>v1.1.4</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="F7" s="3" t="inlineStr">
         <is>
           <t>C2 客户端预测评估:确认手感与回滚稳定性后决定是否默认开启</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>docs/c2-client-prediction-port-plan.md</t>
         </is>
@@ -2008,17 +2077,18 @@
           <t>v1.1.4</t>
         </is>
       </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>公网 IP 动态问题:加 DDNS 或「开服即写 local_ip.txt + 客户端提示」闭环</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr"/>
+      <c r="G8" s="4" t="n"/>
     </row>
     <row r="9" ht="38" customHeight="1">
       <c r="B9" s="3" t="inlineStr">
@@ -2031,17 +2101,18 @@
           <t>v1.1.4</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="F9" s="3" t="inlineStr">
         <is>
           <t>端到端回归:关服后跑整链路探针 + 敌人逻辑冒烟</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Tests/royale_probe.tscn、Tests/enemy_logic_smoke.gd</t>
         </is>
@@ -2050,117 +2121,154 @@
     <row r="10" ht="22" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>企划池</t>
+          <t>下一版计划</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>未定</t>
+          <t>v1.1.4</t>
         </is>
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
+          <t>RoF</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>大乱斗:更多局内事件(空投 / 缩圈 / 击杀播报排行)</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr"/>
-    </row>
-    <row r="11" ht="38" customHeight="1">
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>将大乱斗服务器部分迁移至咕呱蛙的公共服务器中</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="n"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>企划池</t>
+          <t>下一版计划</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>未定</t>
+          <t>v1.1.4</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
+          <t>RoF</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>武器:激光系衍生(穿透 / 持续灼烧 / 扇面)按 LaserWeaponBase 三缝扩展</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr"/>
-    </row>
-    <row r="12" ht="22" customHeight="1">
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>关于部分UI风格化统一问题</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="n"/>
+    </row>
+    <row r="12" ht="38" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>企划池</t>
+          <t>下一版计划</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>未定</t>
+          <t>v1.1.4</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
+          <t>KikuchiH</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>菜单背景主角遇墙的视觉处理</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr"/>
-    </row>
-    <row r="13" ht="22" customHeight="1">
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>修复所有目前有的UI重叠问题</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>可能会在线下会议后在v1.1.5才正式推送</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="38" customHeight="1">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>企划池</t>
+          <t>下一版计划</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>未定</t>
+          <t>v1.1.4</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
+          <t>KikuchiH</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>BGM(Music 总线已留)</t>
-        </is>
-      </c>
-      <c r="F13" s="3" t="inlineStr"/>
-    </row>
-    <row r="14" ht="22" customHeight="1">
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>确认角色卡和武器卡编辑系统彻底可用，新增道具卡编辑系统</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>可能会在线下会议后在v1.1.5才正式推送</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="38" customHeight="1">
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>企划池</t>
+          <t>下一版计划</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>未定</t>
+          <t>v1.1.4</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
+          <t>KikuchiH</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>键位组合键</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr"/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>使用编辑系统实装一名新角色和一把武器，测试完全可用</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>可能会在线下会议后在v1.1.5才正式推送</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="3" t="inlineStr">
@@ -2173,17 +2281,18 @@
           <t>未定</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>小地图 destroyed 砖实时刷新</t>
-        </is>
-      </c>
-      <c r="F15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>大乱斗:更多局内事件(空投 / 缩圈 / 击杀播报排行)</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="n"/>
     </row>
     <row r="16" ht="38" customHeight="1">
       <c r="B16" s="4" t="inlineStr">
@@ -2196,24 +2305,145 @@
           <t>未定</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="4" t="inlineStr">
         <is>
           <t>待办</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>武器:激光系衍生(穿透 / 持续灼烧 / 扇面)按 LaserWeaponBase 三缝扩展</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>企划池</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>未定</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>菜单背景主角遇墙的视觉处理</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>企划池</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>未定</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>BGM(Music 总线已留)</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="n"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>企划池</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>未定</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>键位组合键</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>企划池</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>未定</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>小地图 destroyed 砖实时刷新</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="n"/>
+    </row>
+    <row r="21" ht="38" customHeight="1">
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>企划池</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>未定</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>待办</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>段错误遗留:进图方向约 50% headless 段错误未根治,需带符号引擎抓栈</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr"/>
+      <c r="G21" s="3" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="B4:F16"/>
+  <autoFilter ref="B4:G21"/>
   <mergeCells count="1">
-    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="D5:D16">
+  <conditionalFormatting sqref="E5:E21">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"已完成"</formula>
     </cfRule>
@@ -2222,7 +2452,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="D5:D16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E5:E21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"待办,进行中,已完成"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2236,7 +2466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="B2:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>

</xml_diff>